<commit_message>
Update 718708 - MSCI China A Index .xlsx
</commit_message>
<xml_diff>
--- a/data/718708 - MSCI China A Index .xlsx
+++ b/data/718708 - MSCI China A Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4543" uniqueCount="4542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="4566">
   <si>
     <t>Index Level:</t>
   </si>
@@ -13637,6 +13637,78 @@
   </si>
   <si>
     <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -14022,7 +14094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E4527"/>
+  <dimension ref="A3:E4551"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -50275,6 +50347,198 @@
         <v>2904.70714</v>
       </c>
     </row>
+    <row r="4528" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4528" t="s">
+        <v>4542</v>
+      </c>
+      <c r="B4528">
+        <v>2899.458362</v>
+      </c>
+    </row>
+    <row r="4529" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4529" t="s">
+        <v>4543</v>
+      </c>
+      <c r="B4529">
+        <v>2872.711352</v>
+      </c>
+    </row>
+    <row r="4530" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4530" t="s">
+        <v>4544</v>
+      </c>
+      <c r="B4530">
+        <v>2935.216052</v>
+      </c>
+    </row>
+    <row r="4531" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4531" t="s">
+        <v>4545</v>
+      </c>
+      <c r="B4531">
+        <v>2895.042396</v>
+      </c>
+    </row>
+    <row r="4532" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4532" t="s">
+        <v>4546</v>
+      </c>
+      <c r="B4532">
+        <v>2868.721163</v>
+      </c>
+    </row>
+    <row r="4533" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4533" t="s">
+        <v>4547</v>
+      </c>
+      <c r="B4533">
+        <v>2875.229748</v>
+      </c>
+    </row>
+    <row r="4534" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4534" t="s">
+        <v>4548</v>
+      </c>
+      <c r="B4534">
+        <v>2882.532999</v>
+      </c>
+    </row>
+    <row r="4535" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4535" t="s">
+        <v>4549</v>
+      </c>
+      <c r="B4535">
+        <v>3003.178696</v>
+      </c>
+    </row>
+    <row r="4536" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4536" t="s">
+        <v>4550</v>
+      </c>
+      <c r="B4536">
+        <v>2979.105443</v>
+      </c>
+    </row>
+    <row r="4537" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4537" t="s">
+        <v>4551</v>
+      </c>
+      <c r="B4537">
+        <v>3024.122397</v>
+      </c>
+    </row>
+    <row r="4538" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4538" t="s">
+        <v>4552</v>
+      </c>
+      <c r="B4538">
+        <v>3029.30391</v>
+      </c>
+    </row>
+    <row r="4539" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4539" t="s">
+        <v>4553</v>
+      </c>
+      <c r="B4539">
+        <v>3076.911855</v>
+      </c>
+    </row>
+    <row r="4540" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4540" t="s">
+        <v>4554</v>
+      </c>
+      <c r="B4540">
+        <v>3062.191069</v>
+      </c>
+    </row>
+    <row r="4541" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4541" t="s">
+        <v>4555</v>
+      </c>
+      <c r="B4541">
+        <v>3093.47153</v>
+      </c>
+    </row>
+    <row r="4542" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4542" t="s">
+        <v>4556</v>
+      </c>
+      <c r="B4542">
+        <v>3094.828912</v>
+      </c>
+    </row>
+    <row r="4543" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4543" t="s">
+        <v>4557</v>
+      </c>
+      <c r="B4543">
+        <v>3112.369773</v>
+      </c>
+    </row>
+    <row r="4544" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4544" t="s">
+        <v>4558</v>
+      </c>
+      <c r="B4544">
+        <v>3111.374651</v>
+      </c>
+    </row>
+    <row r="4545" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4545" t="s">
+        <v>4559</v>
+      </c>
+      <c r="B4545">
+        <v>3133.470391</v>
+      </c>
+    </row>
+    <row r="4546" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4546" t="s">
+        <v>4560</v>
+      </c>
+      <c r="B4546">
+        <v>3119.071095</v>
+      </c>
+    </row>
+    <row r="4547" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4547" t="s">
+        <v>4561</v>
+      </c>
+      <c r="B4547">
+        <v>3107.844529</v>
+      </c>
+    </row>
+    <row r="4548" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4548" t="s">
+        <v>4562</v>
+      </c>
+      <c r="B4548">
+        <v>3118.259912</v>
+      </c>
+    </row>
+    <row r="4549" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4549" t="s">
+        <v>4563</v>
+      </c>
+      <c r="B4549">
+        <v>3101.059786</v>
+      </c>
+    </row>
+    <row r="4550" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4550" t="s">
+        <v>4564</v>
+      </c>
+      <c r="B4550">
+        <v>3136.601986</v>
+      </c>
+    </row>
+    <row r="4551" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4551" t="s">
+        <v>4565</v>
+      </c>
+      <c r="B4551">
+        <v>3139.787271</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>